<commit_message>
the structural tests now pass
... still need to update the other tests
</commit_message>
<xml_diff>
--- a/tests/data/structural.xlsx
+++ b/tests/data/structural.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A90BEE-B6E7-4247-AD32-CBE29B53EBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CD020E0-DA8E-544C-BB97-E8F6E05585FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{DE17C082-B7AC-184B-8DE6-41F02A2D59B3}"/>
+    <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{DE17C082-B7AC-184B-8DE6-41F02A2D59B3}"/>
   </bookViews>
   <sheets>
     <sheet name="paige" sheetId="1" r:id="rId1"/>
+    <sheet name="stuff" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>ptid</t>
   </si>
@@ -66,6 +67,12 @@
   </si>
   <si>
     <t>nuh23</t>
+  </si>
+  <si>
+    <t>there's no data on this page</t>
+  </si>
+  <si>
+    <t>just instructions</t>
   </si>
 </sst>
 </file>
@@ -488,4 +495,45 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD31A78B-9673-FE44-A156-788C4FD4356B}">
+  <dimension ref="B2:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B5" s="1"/>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B6" s="1"/>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B7" s="1"/>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B8" s="1"/>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B9" s="1"/>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B10" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>